<commit_message>
docs: lower log lite price
</commit_message>
<xml_diff>
--- a/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
+++ b/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
@@ -263,7 +263,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1,980円/月（税抜案）</t>
+          <t>980円/月（税抜案）</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -273,7 +273,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Log LiteはPremiumより高く見える一方、容量は小さい。Premium対抗ではなく見せ球として説明する</t>
+          <t>Log LiteはPremiumより安く見える一方、容量は小さい。Premium対抗ではなく見せ球として説明する</t>
         </is>
       </c>
     </row>
@@ -295,7 +295,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>23,760円/年（税抜案）</t>
+          <t>11,760円/年（税抜案）</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1000,10 +1000,10 @@
         <v>14220</v>
       </c>
       <c r="D2">
-        <v>1980</v>
+        <v>980</v>
       </c>
       <c r="E2">
-        <v>23760</v>
+        <v>11760</v>
       </c>
       <c r="F2">
         <v>2980</v>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1,980円/月（税抜案）</t>
+          <t>980円/月（税抜案）</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Log Liteの方が高く見える</t>
+          <t>Log Liteの方が安く見える</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">

</xml_diff>

<commit_message>
docs: align log lite caps with notta premium
</commit_message>
<xml_diff>
--- a/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
+++ b/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
@@ -145,7 +145,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Log Liteはログ超過時に停止。超過課金は設定せず、それ以上使いたい場合はkintone Packへの移管を必須にする</t>
+          <t>Log Liteは上限超過時に停止。超過課金は設定せず、それ以上使いたい場合はkintone Packへの移管を必須にする</t>
         </is>
       </c>
     </row>
@@ -157,7 +157,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>現行Log Lite案（月10ログ・1ログ60分・AI要約10回）はNotta Premiumより容量が小さい。Premium対抗ではなく制限付き見せ球として扱う</t>
+          <t>現行Log Lite案（月1,800分・1回5時間・AI要約100回）はNotta Premiumの主要上限に寄せる。価格アンカーとして扱い、kintone連携はPackで差分化する</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Log LiteはPremiumより安く見える一方、容量は小さい。Premium対抗ではなく見せ球として説明する</t>
+          <t>Log LiteはPremiumより安く、主要な利用上限はPremium基準に寄せる。kintone連携はPackで差分化する</t>
         </is>
       </c>
     </row>
@@ -391,7 +391,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>月10ログ x 60分 = 最大600分/月</t>
+          <t>最大1,800分/月</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -401,7 +401,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Log LiteはPremium基準の3分の1。Premium対抗ではなく軽量見せ球</t>
+          <t>Log LiteはPremium基準に合わせ、価格アンカーとして説明する</t>
         </is>
       </c>
     </row>
@@ -423,7 +423,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>60分/ログ</t>
+          <t>5時間/ログ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -433,7 +433,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Premium比較では1回上限の差が目立つ</t>
+          <t>1回上限もPremium基準に合わせる</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10回/月</t>
+          <t>100回/月</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>現行Log Liteの10回はPremiumではなくFree寄りに見える</t>
+          <t>Log LiteもPremium基準の100回/月に寄せる</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ログ超過時の扱い</t>
+          <t>上限超過時の扱い</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10回/月</t>
+          <t>100回/月</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Premium対抗にするなら容量差を埋める。現行案のままならPremium相当とは言わない</t>
+          <t>主要上限はPremium基準に合わせる。kintone連携はPackで差分化する</t>
         </is>
       </c>
     </row>
@@ -1271,17 +1271,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>最大600分/月</t>
+          <t>最大1,800分/月</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Premiumの3分の1</t>
+          <t>Premiumと同等</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Premium比較では劣後。制限付き見せ球として明示</t>
+          <t>Premium比較で見劣りしない上限にする</t>
         </is>
       </c>
     </row>
@@ -1298,17 +1298,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>60分/ログ</t>
+          <t>5時間/ログ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長尺会議で差が出る</t>
+          <t>Premiumと同等</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>用途を短時間ログに限定する</t>
+          <t>1回上限もPremium基準に合わせる</t>
         </is>
       </c>
     </row>
@@ -1325,17 +1325,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10回/月</t>
+          <t>100回/月</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PremiumではなくFree寄りに見える</t>
+          <t>Premiumと同等</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Premium基準なら100回/月を検討。現行案では軽量版として明記</t>
+          <t>要約回数もPremium基準に合わせる</t>
         </is>
       </c>
     </row>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>月10ログ超過で停止。追加課金なし</t>
+          <t>月1,800分または要約100回超過で停止。追加課金なし</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>超過時の利便性より、Pack移管を優先</t>
+          <t>上限超過後はPack移管を優先</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>軽量利用の受け皿</t>
+          <t>Premium基準の1ID見せ球</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Premium比較では劣後しやすい</t>
+          <t>議事録単体の比較には耐えるが、連携価値はPackで差分化</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>

<commit_message>
Salvage additive backup from 2026-06-20
</commit_message>
<xml_diff>
--- a/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
+++ b/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
@@ -145,7 +145,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Log Liteは上限超過時に停止。超過課金は設定せず、それ以上使いたい場合はkintone Packへの移管を必須にする</t>
+          <t>Log Liteはログ超過時に停止。超過課金は設定せず、それ以上使いたい場合はkintone Packへの移管を必須にする</t>
         </is>
       </c>
     </row>
@@ -157,7 +157,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>現行Log Lite案（月1,800分・1回5時間・AI要約100回）はNotta Premiumの主要上限に寄せる。価格アンカーとして扱い、kintone連携はPackで差分化する</t>
+          <t>現行Log Lite案（月10ログ・1ログ60分・AI要約10回）はNotta Premiumより容量が小さい。Premium対抗ではなく制限付き見せ球として扱う</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Log LiteはPremiumより安く、主要な利用上限はPremium基準に寄せる。kintone連携はPackで差分化する</t>
+          <t>Log LiteはPremiumより安く見える一方、容量は小さい。Premium対抗ではなく見せ球として説明する</t>
         </is>
       </c>
     </row>
@@ -391,7 +391,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>最大1,800分/月</t>
+          <t>月10ログ x 60分 = 最大600分/月</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -401,7 +401,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Log LiteはPremium基準に合わせ、価格アンカーとして説明する</t>
+          <t>Log LiteはPremium基準の3分の1。Premium対抗ではなく軽量見せ球</t>
         </is>
       </c>
     </row>
@@ -423,7 +423,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5時間/ログ</t>
+          <t>60分/ログ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -433,7 +433,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1回上限もPremium基準に合わせる</t>
+          <t>Premium比較では1回上限の差が目立つ</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>100回/月</t>
+          <t>10回/月</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Log LiteもPremium基準の100回/月に寄せる</t>
+          <t>現行Log Liteの10回はPremiumではなくFree寄りに見える</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>上限超過時の扱い</t>
+          <t>ログ超過時の扱い</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>100回/月</t>
+          <t>10回/月</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>主要上限はPremium基準に合わせる。kintone連携はPackで差分化する</t>
+          <t>Premium対抗にするなら容量差を埋める。現行案のままならPremium相当とは言わない</t>
         </is>
       </c>
     </row>
@@ -1271,17 +1271,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>最大1,800分/月</t>
+          <t>最大600分/月</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Premiumと同等</t>
+          <t>Premiumの3分の1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Premium比較で見劣りしない上限にする</t>
+          <t>Premium比較では劣後。制限付き見せ球として明示</t>
         </is>
       </c>
     </row>
@@ -1298,17 +1298,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5時間/ログ</t>
+          <t>60分/ログ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Premiumと同等</t>
+          <t>長尺会議で差が出る</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1回上限もPremium基準に合わせる</t>
+          <t>用途を短時間ログに限定する</t>
         </is>
       </c>
     </row>
@@ -1325,17 +1325,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>100回/月</t>
+          <t>10回/月</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Premiumと同等</t>
+          <t>PremiumではなくFree寄りに見える</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>要約回数もPremium基準に合わせる</t>
+          <t>Premium基準なら100回/月を検討。現行案では軽量版として明記</t>
         </is>
       </c>
     </row>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>月1,800分または要約100回超過で停止。追加課金なし</t>
+          <t>月10ログ超過で停止。追加課金なし</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>上限超過後はPack移管を優先</t>
+          <t>超過時の利便性より、Pack移管を優先</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Premium基準の1ID見せ球</t>
+          <t>軽量利用の受け皿</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>議事録単体の比較には耐えるが、連携価値はPackで差分化</t>
+          <t>Premium比較では劣後しやすい</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>

<commit_message>
Additive salvage backup from 2026-06-20
Squash merge additive recovery changes from salvage-20260620-additive.
</commit_message>
<xml_diff>
--- a/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
+++ b/deck-system/decks/umee-sbcs-kintone-plan/exports/notta-premium-frontagent-comparison.xlsx
@@ -145,7 +145,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Log Liteは上限超過時に停止。超過課金は設定せず、それ以上使いたい場合はkintone Packへの移管を必須にする</t>
+          <t>Log Liteはログ超過時に停止。超過課金は設定せず、それ以上使いたい場合はkintone Packへの移管を必須にする</t>
         </is>
       </c>
     </row>
@@ -157,7 +157,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>現行Log Lite案（月1,800分・1回5時間・AI要約100回）はNotta Premiumの主要上限に寄せる。価格アンカーとして扱い、kintone連携はPackで差分化する</t>
+          <t>現行Log Lite案（月10ログ・1ログ60分・AI要約10回）はNotta Premiumより容量が小さい。Premium対抗ではなく制限付き見せ球として扱う</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Log LiteはPremiumより安く、主要な利用上限はPremium基準に寄せる。kintone連携はPackで差分化する</t>
+          <t>Log LiteはPremiumより安く見える一方、容量は小さい。Premium対抗ではなく見せ球として説明する</t>
         </is>
       </c>
     </row>
@@ -391,7 +391,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>最大1,800分/月</t>
+          <t>月10ログ x 60分 = 最大600分/月</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -401,7 +401,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Log LiteはPremium基準に合わせ、価格アンカーとして説明する</t>
+          <t>Log LiteはPremium基準の3分の1。Premium対抗ではなく軽量見せ球</t>
         </is>
       </c>
     </row>
@@ -423,7 +423,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5時間/ログ</t>
+          <t>60分/ログ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -433,7 +433,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1回上限もPremium基準に合わせる</t>
+          <t>Premium比較では1回上限の差が目立つ</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>100回/月</t>
+          <t>10回/月</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Log LiteもPremium基準の100回/月に寄せる</t>
+          <t>現行Log Liteの10回はPremiumではなくFree寄りに見える</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>上限超過時の扱い</t>
+          <t>ログ超過時の扱い</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>100回/月</t>
+          <t>10回/月</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>主要上限はPremium基準に合わせる。kintone連携はPackで差分化する</t>
+          <t>Premium対抗にするなら容量差を埋める。現行案のままならPremium相当とは言わない</t>
         </is>
       </c>
     </row>
@@ -1271,17 +1271,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>最大1,800分/月</t>
+          <t>最大600分/月</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Premiumと同等</t>
+          <t>Premiumの3分の1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Premium比較で見劣りしない上限にする</t>
+          <t>Premium比較では劣後。制限付き見せ球として明示</t>
         </is>
       </c>
     </row>
@@ -1298,17 +1298,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5時間/ログ</t>
+          <t>60分/ログ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Premiumと同等</t>
+          <t>長尺会議で差が出る</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1回上限もPremium基準に合わせる</t>
+          <t>用途を短時間ログに限定する</t>
         </is>
       </c>
     </row>
@@ -1325,17 +1325,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>100回/月</t>
+          <t>10回/月</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Premiumと同等</t>
+          <t>PremiumではなくFree寄りに見える</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>要約回数もPremium基準に合わせる</t>
+          <t>Premium基準なら100回/月を検討。現行案では軽量版として明記</t>
         </is>
       </c>
     </row>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>月1,800分または要約100回超過で停止。追加課金なし</t>
+          <t>月10ログ超過で停止。追加課金なし</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>上限超過後はPack移管を優先</t>
+          <t>超過時の利便性より、Pack移管を優先</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Premium基準の1ID見せ球</t>
+          <t>軽量利用の受け皿</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>議事録単体の比較には耐えるが、連携価値はPackで差分化</t>
+          <t>Premium比較では劣後しやすい</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>